<commit_message>
fix(upload): não setar valor_unitario/valor_total (colunas geradas)
</commit_message>
<xml_diff>
--- a/docs/Cronograma Fisico Financeiro - upload base.xlsx
+++ b/docs/Cronograma Fisico Financeiro - upload base.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b73f7ac4adb68b79/APP-GESTAO-CONTRATO/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="107" documentId="11_44BB8124A3813D6CE061023760305AB482D18CB9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0CBBD25-0FC7-46A3-AD2A-CEC428CEA8B2}"/>
+  <xr:revisionPtr revIDLastSave="109" documentId="11_44BB8124A3813D6CE061023760305AB482D18CB9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C385F0BE-8F84-4676-93A3-E6BC1B30BC16}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3269,91 +3269,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentagem" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="23">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="11">
     <dxf>
       <fill>
         <patternFill>
@@ -29165,7 +29081,7 @@
         <v>5.5555555555555552E-2</v>
       </c>
       <c r="AB406" s="20">
-        <f t="shared" ref="V406:AD407" si="61">1/18</f>
+        <f t="shared" ref="V406:AC407" si="61">1/18</f>
         <v>5.5555555555555552E-2</v>
       </c>
       <c r="AC406" s="20">

</xml_diff>